<commit_message>
daily auto-refresh 2026-09-24 15:01
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -518,16 +518,16 @@
         <v>4</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -907,10 +907,10 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>1</v>
@@ -1838,10 +1838,10 @@
         <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
         <v>4</v>
@@ -4294,10 +4294,10 @@
         <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -5127,10 +5127,10 @@
         <v>0</v>
       </c>
       <c r="I96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K96" t="n">
         <v>0</v>
@@ -7972,10 +7972,10 @@
         <v>5</v>
       </c>
       <c r="J154" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K154" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L154" t="n">
         <v>0</v>
@@ -8211,7 +8211,7 @@
         <v>8</v>
       </c>
       <c r="H159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I159" t="n">
         <v>3</v>
@@ -8220,7 +8220,7 @@
         <v>0</v>
       </c>
       <c r="K159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L159" t="n">
         <v>0</v>
@@ -8263,10 +8263,10 @@
         <v>1</v>
       </c>
       <c r="I160" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J160" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K160" t="n">
         <v>0</v>
@@ -9776,10 +9776,10 @@
         <v>13</v>
       </c>
       <c r="G191" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H191" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I191" t="n">
         <v>2</v>
@@ -10315,10 +10315,10 @@
         <v>25</v>
       </c>
       <c r="G202" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H202" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I202" t="n">
         <v>17</v>
@@ -11589,10 +11589,10 @@
         <v>3</v>
       </c>
       <c r="G228" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H228" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I228" t="n">
         <v>5</v>
@@ -11843,10 +11843,10 @@
         <v>3</v>
       </c>
       <c r="J233" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K233" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L233" t="n">
         <v>0</v>
@@ -13007,16 +13007,16 @@
         <v>2</v>
       </c>
       <c r="F257" t="n">
+        <v>7</v>
+      </c>
+      <c r="G257" t="n">
+        <v>28</v>
+      </c>
+      <c r="H257" t="n">
         <v>6</v>
       </c>
-      <c r="G257" t="n">
-        <v>29</v>
-      </c>
-      <c r="H257" t="n">
-        <v>5</v>
-      </c>
       <c r="I257" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J257" t="n">
         <v>0</v>
@@ -13356,10 +13356,10 @@
         <v>13</v>
       </c>
       <c r="H264" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I264" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J264" t="n">
         <v>0</v>
@@ -13509,10 +13509,10 @@
         <v>3</v>
       </c>
       <c r="J267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K267" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L267" t="n">
         <v>3</v>
@@ -14140,10 +14140,10 @@
         <v>8</v>
       </c>
       <c r="H280" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I280" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J280" t="n">
         <v>4</v>
@@ -15267,10 +15267,10 @@
         <v>90</v>
       </c>
       <c r="H303" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I303" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J303" t="n">
         <v>3</v>
@@ -15561,10 +15561,10 @@
         <v>24</v>
       </c>
       <c r="H309" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I309" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J309" t="n">
         <v>3</v>
@@ -15754,10 +15754,10 @@
         <v>31</v>
       </c>
       <c r="G313" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H313" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I313" t="n">
         <v>12</v>
@@ -15950,10 +15950,10 @@
         <v>8</v>
       </c>
       <c r="G317" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H317" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I317" t="n">
         <v>7</v>
@@ -16394,10 +16394,10 @@
         <v>6</v>
       </c>
       <c r="H326" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I326" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J326" t="n">
         <v>0</v>
@@ -16685,10 +16685,10 @@
         <v>4</v>
       </c>
       <c r="G332" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H332" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I332" t="n">
         <v>3</v>
@@ -16734,10 +16734,10 @@
         <v>2</v>
       </c>
       <c r="G333" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H333" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17570,10 +17570,10 @@
         <v>1</v>
       </c>
       <c r="H350" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I350" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J350" t="n">
         <v>0</v>
@@ -17601,7 +17601,7 @@
         </is>
       </c>
       <c r="B351" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C351" t="n">
         <v>0</v>
@@ -17619,10 +17619,10 @@
         <v>15</v>
       </c>
       <c r="H351" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I351" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J351" t="n">
         <v>0</v>
@@ -17631,7 +17631,7 @@
         <v>1</v>
       </c>
       <c r="L351" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M351" t="n">
         <v>46</v>
@@ -17708,7 +17708,7 @@
         <v>0</v>
       </c>
       <c r="E353" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F353" t="n">
         <v>1</v>
@@ -17729,7 +17729,7 @@
         <v>1</v>
       </c>
       <c r="L353" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M353" t="n">
         <v>44</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-01 15:34
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -3109,10 +3109,10 @@
         <v>2</v>
       </c>
       <c r="F55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H55" t="n">
         <v>2</v>
@@ -7911,10 +7911,10 @@
         <v>4</v>
       </c>
       <c r="F153" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G153" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H153" t="n">
         <v>4</v>
@@ -7960,10 +7960,10 @@
         <v>10</v>
       </c>
       <c r="F154" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G154" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H154" t="n">
         <v>7</v>
@@ -8845,10 +8845,10 @@
         <v>12</v>
       </c>
       <c r="G172" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H172" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I172" t="n">
         <v>2</v>
@@ -11298,10 +11298,10 @@
         <v>18</v>
       </c>
       <c r="H222" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I222" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J222" t="n">
         <v>0</v>
@@ -12076,10 +12076,10 @@
         <v>25</v>
       </c>
       <c r="F238" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G238" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H238" t="n">
         <v>5</v>
@@ -12125,10 +12125,10 @@
         <v>0</v>
       </c>
       <c r="F239" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G239" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H239" t="n">
         <v>0</v>
@@ -13497,10 +13497,10 @@
         <v>25</v>
       </c>
       <c r="F267" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G267" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H267" t="n">
         <v>6</v>
@@ -13549,10 +13549,10 @@
         <v>11</v>
       </c>
       <c r="G268" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H268" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I268" t="n">
         <v>2</v>
@@ -13690,13 +13690,13 @@
         <v>3</v>
       </c>
       <c r="E271" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F271" t="n">
         <v>11</v>
       </c>
       <c r="G271" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H271" t="n">
         <v>1</v>
@@ -13889,13 +13889,13 @@
         <v>26</v>
       </c>
       <c r="F275" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G275" t="n">
         <v>16</v>
       </c>
       <c r="H275" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I275" t="n">
         <v>2</v>
@@ -14526,10 +14526,10 @@
         <v>1</v>
       </c>
       <c r="F288" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G288" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H288" t="n">
         <v>8</v>
@@ -14918,10 +14918,10 @@
         <v>30</v>
       </c>
       <c r="F296" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G296" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H296" t="n">
         <v>3</v>
@@ -15754,10 +15754,10 @@
         <v>31</v>
       </c>
       <c r="G313" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H313" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I313" t="n">
         <v>12</v>
@@ -15800,10 +15800,10 @@
         <v>27</v>
       </c>
       <c r="F314" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G314" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H314" t="n">
         <v>9</v>
@@ -16593,10 +16593,10 @@
         <v>9</v>
       </c>
       <c r="I330" t="n">
+        <v>3</v>
+      </c>
+      <c r="J330" t="n">
         <v>4</v>
-      </c>
-      <c r="J330" t="n">
-        <v>3</v>
       </c>
       <c r="K330" t="n">
         <v>1</v>
@@ -16734,10 +16734,10 @@
         <v>2</v>
       </c>
       <c r="G333" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H333" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -16979,7 +16979,7 @@
         <v>3</v>
       </c>
       <c r="G338" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H338" t="n">
         <v>9</v>
@@ -16994,7 +16994,7 @@
         <v>1</v>
       </c>
       <c r="L338" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M338" t="n">
         <v>49</v>
@@ -17086,13 +17086,13 @@
         <v>0</v>
       </c>
       <c r="J340" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K340" t="n">
         <v>0</v>
       </c>
       <c r="L340" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M340" t="n">
         <v>12</v>
@@ -17273,10 +17273,10 @@
         <v>6</v>
       </c>
       <c r="G344" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H344" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I344" t="n">
         <v>6</v>
@@ -17714,22 +17714,22 @@
         <v>1</v>
       </c>
       <c r="G353" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H353" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I353" t="n">
         <v>3</v>
       </c>
       <c r="J353" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K353" t="n">
         <v>1</v>
       </c>
       <c r="L353" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M353" t="n">
         <v>44</v>
@@ -18008,13 +18008,13 @@
         <v>8</v>
       </c>
       <c r="G359" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H359" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I359" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J359" t="n">
         <v>1</v>
@@ -18023,7 +18023,7 @@
         <v>0</v>
       </c>
       <c r="L359" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="M359" t="n">
         <v>92</v>
@@ -18054,25 +18054,25 @@
         <v>1</v>
       </c>
       <c r="F360" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G360" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H360" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I360" t="n">
         <v>5</v>
       </c>
       <c r="J360" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K360" t="n">
         <v>0</v>
       </c>
       <c r="L360" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="M360" t="n">
         <v>47</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-07 16:35
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -9874,7 +9874,7 @@
         <v>11</v>
       </c>
       <c r="G193" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H193" t="n">
         <v>2</v>
@@ -9889,7 +9889,7 @@
         <v>2</v>
       </c>
       <c r="L193" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M193" t="n">
         <v>82</v>
@@ -10006,25 +10006,25 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C196" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D196" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E196" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F196" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G196" t="n">
         <v>17</v>
       </c>
       <c r="H196" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I196" t="n">
         <v>4</v>
@@ -10036,7 +10036,7 @@
         <v>0</v>
       </c>
       <c r="L196" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M196" t="n">
         <v>103</v>
@@ -10055,7 +10055,7 @@
         </is>
       </c>
       <c r="B197" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C197" t="n">
         <v>5</v>
@@ -10085,7 +10085,7 @@
         <v>1</v>
       </c>
       <c r="L197" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M197" t="n">
         <v>63</v>
@@ -10104,7 +10104,7 @@
         </is>
       </c>
       <c r="B198" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C198" t="n">
         <v>9</v>
@@ -10119,7 +10119,7 @@
         <v>8</v>
       </c>
       <c r="G198" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H198" t="n">
         <v>1</v>
@@ -10134,7 +10134,7 @@
         <v>0</v>
       </c>
       <c r="L198" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M198" t="n">
         <v>62</v>
@@ -10162,14 +10162,14 @@
         <v>9</v>
       </c>
       <c r="E199" t="n">
+        <v>13</v>
+      </c>
+      <c r="F199" t="n">
+        <v>3</v>
+      </c>
+      <c r="G199" t="n">
         <v>11</v>
       </c>
-      <c r="F199" t="n">
-        <v>3</v>
-      </c>
-      <c r="G199" t="n">
-        <v>10</v>
-      </c>
       <c r="H199" t="n">
         <v>1</v>
       </c>
@@ -10183,7 +10183,7 @@
         <v>0</v>
       </c>
       <c r="L199" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M199" t="n">
         <v>58</v>
@@ -10214,7 +10214,7 @@
         <v>11</v>
       </c>
       <c r="F200" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G200" t="n">
         <v>3</v>
@@ -10232,7 +10232,7 @@
         <v>0</v>
       </c>
       <c r="L200" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M200" t="n">
         <v>44</v>
@@ -10300,16 +10300,16 @@
         </is>
       </c>
       <c r="B202" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C202" t="n">
         <v>8</v>
       </c>
       <c r="D202" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E202" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F202" t="n">
         <v>25</v>
@@ -10318,10 +10318,10 @@
         <v>36</v>
       </c>
       <c r="H202" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I202" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J202" t="n">
         <v>6</v>
@@ -10330,7 +10330,7 @@
         <v>3</v>
       </c>
       <c r="L202" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M202" t="n">
         <v>181</v>
@@ -10422,13 +10422,13 @@
         <v>4</v>
       </c>
       <c r="J204" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K204" t="n">
         <v>0</v>
       </c>
       <c r="L204" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M204" t="n">
         <v>103</v>
@@ -10508,7 +10508,7 @@
         <v>1</v>
       </c>
       <c r="F206" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G206" t="n">
         <v>8</v>
@@ -10526,7 +10526,7 @@
         <v>2</v>
       </c>
       <c r="L206" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M206" t="n">
         <v>25</v>
@@ -10664,7 +10664,7 @@
         <v>2</v>
       </c>
       <c r="I209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J209" t="n">
         <v>0</v>
@@ -10673,7 +10673,7 @@
         <v>0</v>
       </c>
       <c r="L209" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M209" t="n">
         <v>15</v>
@@ -10805,7 +10805,7 @@
         <v>4</v>
       </c>
       <c r="G212" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H212" t="n">
         <v>0</v>
@@ -10820,7 +10820,7 @@
         <v>0</v>
       </c>
       <c r="L212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M212" t="n">
         <v>20</v>
@@ -10848,7 +10848,7 @@
         <v>2</v>
       </c>
       <c r="E213" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F213" t="n">
         <v>3</v>
@@ -10869,7 +10869,7 @@
         <v>0</v>
       </c>
       <c r="L213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M213" t="n">
         <v>17</v>
@@ -11007,7 +11007,7 @@
         <v>3</v>
       </c>
       <c r="I216" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J216" t="n">
         <v>2</v>
@@ -11016,7 +11016,7 @@
         <v>1</v>
       </c>
       <c r="L216" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M216" t="n">
         <v>27</v>
@@ -11093,10 +11093,10 @@
         <v>2</v>
       </c>
       <c r="E218" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F218" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G218" t="n">
         <v>13</v>
@@ -11114,7 +11114,7 @@
         <v>0</v>
       </c>
       <c r="L218" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M218" t="n">
         <v>53</v>
@@ -11142,7 +11142,7 @@
         <v>2</v>
       </c>
       <c r="E219" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F219" t="n">
         <v>7</v>
@@ -11163,7 +11163,7 @@
         <v>1</v>
       </c>
       <c r="L219" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M219" t="n">
         <v>33</v>
@@ -11295,7 +11295,7 @@
         <v>5</v>
       </c>
       <c r="G222" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H222" t="n">
         <v>7</v>
@@ -11310,7 +11310,7 @@
         <v>1</v>
       </c>
       <c r="L222" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M222" t="n">
         <v>59</v>
@@ -11338,10 +11338,10 @@
         <v>1</v>
       </c>
       <c r="E223" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F223" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G223" t="n">
         <v>8</v>
@@ -11359,7 +11359,7 @@
         <v>0</v>
       </c>
       <c r="L223" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M223" t="n">
         <v>29</v>
@@ -11402,13 +11402,13 @@
         <v>2</v>
       </c>
       <c r="J224" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K224" t="n">
         <v>1</v>
       </c>
       <c r="L224" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M224" t="n">
         <v>25</v>
@@ -11482,7 +11482,7 @@
         <v>3</v>
       </c>
       <c r="D226" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E226" t="n">
         <v>7</v>
@@ -11506,7 +11506,7 @@
         <v>0</v>
       </c>
       <c r="L226" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M226" t="n">
         <v>23</v>
@@ -11681,7 +11681,7 @@
         <v>0</v>
       </c>
       <c r="E230" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F230" t="n">
         <v>4</v>
@@ -11702,7 +11702,7 @@
         <v>0</v>
       </c>
       <c r="L230" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M230" t="n">
         <v>38</v>
@@ -11733,7 +11733,7 @@
         <v>6</v>
       </c>
       <c r="F231" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G231" t="n">
         <v>30</v>
@@ -11751,7 +11751,7 @@
         <v>1</v>
       </c>
       <c r="L231" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M231" t="n">
         <v>65</v>
@@ -11825,13 +11825,13 @@
         <v>1</v>
       </c>
       <c r="D233" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E233" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F233" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G233" t="n">
         <v>38</v>
@@ -11849,7 +11849,7 @@
         <v>0</v>
       </c>
       <c r="L233" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M233" t="n">
         <v>86</v>
@@ -11880,7 +11880,7 @@
         <v>8</v>
       </c>
       <c r="F234" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G234" t="n">
         <v>7</v>
@@ -11898,7 +11898,7 @@
         <v>1</v>
       </c>
       <c r="L234" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M234" t="n">
         <v>50</v>
@@ -11972,16 +11972,16 @@
         <v>4</v>
       </c>
       <c r="D236" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E236" t="n">
         <v>37</v>
       </c>
       <c r="F236" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G236" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H236" t="n">
         <v>14</v>
@@ -11996,7 +11996,7 @@
         <v>0</v>
       </c>
       <c r="L236" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M236" t="n">
         <v>187</v>
@@ -12018,7 +12018,7 @@
         <v>5</v>
       </c>
       <c r="C237" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D237" t="n">
         <v>6</v>
@@ -12027,7 +12027,7 @@
         <v>16</v>
       </c>
       <c r="F237" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G237" t="n">
         <v>30</v>
@@ -12045,7 +12045,7 @@
         <v>0</v>
       </c>
       <c r="L237" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M237" t="n">
         <v>86</v>
@@ -12067,10 +12067,10 @@
         <v>8</v>
       </c>
       <c r="C238" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D238" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E238" t="n">
         <v>25</v>
@@ -12094,7 +12094,7 @@
         <v>0</v>
       </c>
       <c r="L238" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M238" t="n">
         <v>120</v>
@@ -12168,13 +12168,13 @@
         <v>5</v>
       </c>
       <c r="D240" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E240" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F240" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G240" t="n">
         <v>65</v>
@@ -12183,7 +12183,7 @@
         <v>8</v>
       </c>
       <c r="I240" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J240" t="n">
         <v>0</v>
@@ -12192,7 +12192,7 @@
         <v>2</v>
       </c>
       <c r="L240" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M240" t="n">
         <v>149</v>
@@ -12220,13 +12220,13 @@
         <v>9</v>
       </c>
       <c r="E241" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F241" t="n">
         <v>14</v>
       </c>
       <c r="G241" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H241" t="n">
         <v>0</v>
@@ -12241,7 +12241,7 @@
         <v>0</v>
       </c>
       <c r="L241" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M241" t="n">
         <v>65</v>
@@ -12263,16 +12263,16 @@
         <v>1</v>
       </c>
       <c r="C242" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D242" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E242" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F242" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G242" t="n">
         <v>20</v>
@@ -12290,7 +12290,7 @@
         <v>1</v>
       </c>
       <c r="L242" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M242" t="n">
         <v>71</v>
@@ -12456,16 +12456,16 @@
         </is>
       </c>
       <c r="B246" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C246" t="n">
         <v>4</v>
       </c>
       <c r="D246" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E246" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F246" t="n">
         <v>22</v>
@@ -12477,7 +12477,7 @@
         <v>11</v>
       </c>
       <c r="I246" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J246" t="n">
         <v>3</v>
@@ -12486,7 +12486,7 @@
         <v>1</v>
       </c>
       <c r="L246" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M246" t="n">
         <v>175</v>
@@ -12511,7 +12511,7 @@
         <v>1</v>
       </c>
       <c r="D247" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E247" t="n">
         <v>4</v>
@@ -12535,7 +12535,7 @@
         <v>0</v>
       </c>
       <c r="L247" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M247" t="n">
         <v>43</v>
@@ -12615,7 +12615,7 @@
         <v>10</v>
       </c>
       <c r="F249" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G249" t="n">
         <v>26</v>
@@ -12633,7 +12633,7 @@
         <v>1</v>
       </c>
       <c r="L249" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M249" t="n">
         <v>59</v>
@@ -12652,7 +12652,7 @@
         </is>
       </c>
       <c r="B250" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C250" t="n">
         <v>0</v>
@@ -12661,7 +12661,7 @@
         <v>0</v>
       </c>
       <c r="E250" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F250" t="n">
         <v>3</v>
@@ -12682,7 +12682,7 @@
         <v>1</v>
       </c>
       <c r="L250" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M250" t="n">
         <v>38</v>
@@ -12869,16 +12869,16 @@
         <v>12</v>
       </c>
       <c r="I254" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J254" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K254" t="n">
         <v>1</v>
       </c>
       <c r="L254" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M254" t="n">
         <v>50</v>
@@ -12897,13 +12897,13 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C255" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D255" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E255" t="n">
         <v>29</v>
@@ -12927,7 +12927,7 @@
         <v>1</v>
       </c>
       <c r="L255" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M255" t="n">
         <v>144</v>
@@ -12946,7 +12946,7 @@
         </is>
       </c>
       <c r="B256" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C256" t="n">
         <v>19</v>
@@ -12976,7 +12976,7 @@
         <v>1</v>
       </c>
       <c r="L256" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M256" t="n">
         <v>222</v>
@@ -13142,10 +13142,10 @@
         </is>
       </c>
       <c r="B260" t="n">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C260" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D260" t="n">
         <v>27</v>
@@ -13157,7 +13157,7 @@
         <v>29</v>
       </c>
       <c r="G260" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H260" t="n">
         <v>18</v>
@@ -13172,7 +13172,7 @@
         <v>3</v>
       </c>
       <c r="L260" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="M260" t="n">
         <v>289</v>
@@ -13191,19 +13191,19 @@
         </is>
       </c>
       <c r="B261" t="n">
-        <v>766</v>
+        <v>797</v>
       </c>
       <c r="C261" t="n">
+        <v>82</v>
+      </c>
+      <c r="D261" t="n">
         <v>80</v>
       </c>
-      <c r="D261" t="n">
-        <v>75</v>
-      </c>
       <c r="E261" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F261" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G261" t="n">
         <v>45</v>
@@ -13221,7 +13221,7 @@
         <v>0</v>
       </c>
       <c r="L261" t="n">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="M261" t="n">
         <v>1160</v>
@@ -13240,19 +13240,19 @@
         </is>
       </c>
       <c r="B262" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C262" t="n">
         <v>18</v>
       </c>
       <c r="D262" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E262" t="n">
         <v>13</v>
       </c>
       <c r="F262" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G262" t="n">
         <v>15</v>
@@ -13261,7 +13261,7 @@
         <v>1</v>
       </c>
       <c r="I262" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J262" t="n">
         <v>0</v>
@@ -13270,7 +13270,7 @@
         <v>1</v>
       </c>
       <c r="L262" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="M262" t="n">
         <v>157</v>
@@ -13289,7 +13289,7 @@
         </is>
       </c>
       <c r="B263" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C263" t="n">
         <v>12</v>
@@ -13319,7 +13319,7 @@
         <v>0</v>
       </c>
       <c r="L263" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M263" t="n">
         <v>171</v>
@@ -13338,7 +13338,7 @@
         </is>
       </c>
       <c r="B264" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C264" t="n">
         <v>13</v>
@@ -13347,7 +13347,7 @@
         <v>13</v>
       </c>
       <c r="E264" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F264" t="n">
         <v>8</v>
@@ -13368,7 +13368,7 @@
         <v>1</v>
       </c>
       <c r="L264" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M264" t="n">
         <v>189</v>
@@ -13387,7 +13387,7 @@
         </is>
       </c>
       <c r="B265" t="n">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C265" t="n">
         <v>11</v>
@@ -13396,7 +13396,7 @@
         <v>25</v>
       </c>
       <c r="E265" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F265" t="n">
         <v>18</v>
@@ -13417,7 +13417,7 @@
         <v>0</v>
       </c>
       <c r="L265" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M265" t="n">
         <v>268</v>
@@ -13494,13 +13494,13 @@
         <v>7</v>
       </c>
       <c r="E267" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F267" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G267" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H267" t="n">
         <v>6</v>
@@ -13515,7 +13515,7 @@
         <v>0</v>
       </c>
       <c r="L267" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M267" t="n">
         <v>131</v>
@@ -13534,7 +13534,7 @@
         </is>
       </c>
       <c r="B268" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C268" t="n">
         <v>1</v>
@@ -13564,7 +13564,7 @@
         <v>1</v>
       </c>
       <c r="L268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M268" t="n">
         <v>66</v>
@@ -13696,7 +13696,7 @@
         <v>11</v>
       </c>
       <c r="G271" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H271" t="n">
         <v>1</v>
@@ -13711,7 +13711,7 @@
         <v>0</v>
       </c>
       <c r="L271" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M271" t="n">
         <v>49</v>
@@ -13779,7 +13779,7 @@
         </is>
       </c>
       <c r="B273" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C273" t="n">
         <v>0</v>
@@ -13809,7 +13809,7 @@
         <v>0</v>
       </c>
       <c r="L273" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M273" t="n">
         <v>29</v>
@@ -13828,7 +13828,7 @@
         </is>
       </c>
       <c r="B274" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C274" t="n">
         <v>6</v>
@@ -13840,13 +13840,13 @@
         <v>14</v>
       </c>
       <c r="F274" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G274" t="n">
         <v>29</v>
       </c>
       <c r="H274" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I274" t="n">
         <v>4</v>
@@ -13858,7 +13858,7 @@
         <v>0</v>
       </c>
       <c r="L274" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M274" t="n">
         <v>228</v>
@@ -13877,13 +13877,13 @@
         </is>
       </c>
       <c r="B275" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C275" t="n">
         <v>12</v>
       </c>
       <c r="D275" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E275" t="n">
         <v>26</v>
@@ -13907,7 +13907,7 @@
         <v>1</v>
       </c>
       <c r="L275" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="M275" t="n">
         <v>269</v>
@@ -13935,19 +13935,19 @@
         <v>10</v>
       </c>
       <c r="E276" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F276" t="n">
         <v>10</v>
       </c>
       <c r="G276" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H276" t="n">
         <v>4</v>
       </c>
       <c r="I276" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J276" t="n">
         <v>1</v>
@@ -13956,7 +13956,7 @@
         <v>0</v>
       </c>
       <c r="L276" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="M276" t="n">
         <v>85</v>
@@ -13990,7 +13990,7 @@
         <v>8</v>
       </c>
       <c r="G277" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H277" t="n">
         <v>2</v>
@@ -14005,7 +14005,7 @@
         <v>0</v>
       </c>
       <c r="L277" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M277" t="n">
         <v>100</v>
@@ -14122,7 +14122,7 @@
         </is>
       </c>
       <c r="B280" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C280" t="n">
         <v>2</v>
@@ -14131,7 +14131,7 @@
         <v>8</v>
       </c>
       <c r="E280" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F280" t="n">
         <v>3</v>
@@ -14143,7 +14143,7 @@
         <v>3</v>
       </c>
       <c r="I280" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J280" t="n">
         <v>4</v>
@@ -14152,7 +14152,7 @@
         <v>0</v>
       </c>
       <c r="L280" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="M280" t="n">
         <v>140</v>
@@ -14171,7 +14171,7 @@
         </is>
       </c>
       <c r="B281" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C281" t="n">
         <v>12</v>
@@ -14192,7 +14192,7 @@
         <v>1</v>
       </c>
       <c r="I281" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J281" t="n">
         <v>1</v>
@@ -14201,7 +14201,7 @@
         <v>2</v>
       </c>
       <c r="L281" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="M281" t="n">
         <v>155</v>
@@ -14223,7 +14223,7 @@
         <v>8</v>
       </c>
       <c r="C282" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D282" t="n">
         <v>10</v>
@@ -14250,7 +14250,7 @@
         <v>0</v>
       </c>
       <c r="L282" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M282" t="n">
         <v>96</v>
@@ -14324,7 +14324,7 @@
         <v>0</v>
       </c>
       <c r="D284" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E284" t="n">
         <v>22</v>
@@ -14348,7 +14348,7 @@
         <v>1</v>
       </c>
       <c r="L284" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M284" t="n">
         <v>94</v>
@@ -14382,7 +14382,7 @@
         <v>17</v>
       </c>
       <c r="G285" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H285" t="n">
         <v>2</v>
@@ -14397,7 +14397,7 @@
         <v>0</v>
       </c>
       <c r="L285" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M285" t="n">
         <v>117</v>
@@ -14416,19 +14416,19 @@
         </is>
       </c>
       <c r="B286" t="n">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C286" t="n">
         <v>13</v>
       </c>
       <c r="D286" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E286" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F286" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G286" t="n">
         <v>12</v>
@@ -14440,13 +14440,13 @@
         <v>3</v>
       </c>
       <c r="J286" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K286" t="n">
         <v>1</v>
       </c>
       <c r="L286" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="M286" t="n">
         <v>291</v>
@@ -14563,7 +14563,7 @@
         </is>
       </c>
       <c r="B289" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C289" t="n">
         <v>1</v>
@@ -14593,7 +14593,7 @@
         <v>1</v>
       </c>
       <c r="L289" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M289" t="n">
         <v>100</v>
@@ -14618,7 +14618,7 @@
         <v>11</v>
       </c>
       <c r="D290" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E290" t="n">
         <v>20</v>
@@ -14642,7 +14642,7 @@
         <v>1</v>
       </c>
       <c r="L290" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M290" t="n">
         <v>302</v>
@@ -14664,13 +14664,13 @@
         <v>46</v>
       </c>
       <c r="C291" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D291" t="n">
         <v>12</v>
       </c>
       <c r="E291" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F291" t="n">
         <v>11</v>
@@ -14691,7 +14691,7 @@
         <v>1</v>
       </c>
       <c r="L291" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M291" t="n">
         <v>122</v>
@@ -14857,22 +14857,22 @@
         </is>
       </c>
       <c r="B295" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C295" t="n">
         <v>1</v>
       </c>
       <c r="D295" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E295" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F295" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G295" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H295" t="n">
         <v>7</v>
@@ -14887,7 +14887,7 @@
         <v>0</v>
       </c>
       <c r="L295" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="M295" t="n">
         <v>134</v>
@@ -14906,13 +14906,13 @@
         </is>
       </c>
       <c r="B296" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C296" t="n">
         <v>1</v>
       </c>
       <c r="D296" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E296" t="n">
         <v>29</v>
@@ -14936,7 +14936,7 @@
         <v>0</v>
       </c>
       <c r="L296" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="M296" t="n">
         <v>122</v>
@@ -15368,7 +15368,7 @@
         <v>7</v>
       </c>
       <c r="I305" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J305" t="n">
         <v>3</v>
@@ -15377,7 +15377,7 @@
         <v>0</v>
       </c>
       <c r="L305" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M305" t="n">
         <v>72</v>
@@ -15405,7 +15405,7 @@
         <v>4</v>
       </c>
       <c r="E306" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F306" t="n">
         <v>12</v>
@@ -15426,7 +15426,7 @@
         <v>2</v>
       </c>
       <c r="L306" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M306" t="n">
         <v>78</v>
@@ -15604,7 +15604,7 @@
         <v>7</v>
       </c>
       <c r="F310" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G310" t="n">
         <v>71</v>
@@ -15622,7 +15622,7 @@
         <v>0</v>
       </c>
       <c r="L310" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M310" t="n">
         <v>109</v>
@@ -15702,10 +15702,10 @@
         <v>22</v>
       </c>
       <c r="F312" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G312" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H312" t="n">
         <v>13</v>
@@ -15720,7 +15720,7 @@
         <v>1</v>
       </c>
       <c r="L312" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M312" t="n">
         <v>149</v>
@@ -15751,10 +15751,10 @@
         <v>34</v>
       </c>
       <c r="F313" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G313" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H313" t="n">
         <v>18</v>
@@ -15769,7 +15769,7 @@
         <v>1</v>
       </c>
       <c r="L313" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M313" t="n">
         <v>232</v>
@@ -15791,19 +15791,19 @@
         <v>12</v>
       </c>
       <c r="C314" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D314" t="n">
         <v>16</v>
       </c>
       <c r="E314" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F314" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G314" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H314" t="n">
         <v>9</v>
@@ -15818,7 +15818,7 @@
         <v>0</v>
       </c>
       <c r="L314" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="M314" t="n">
         <v>210</v>
@@ -15990,10 +15990,10 @@
         <v>4</v>
       </c>
       <c r="D318" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E318" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F318" t="n">
         <v>9</v>
@@ -16014,7 +16014,7 @@
         <v>0</v>
       </c>
       <c r="L318" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="M318" t="n">
         <v>91</v>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="E322" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F322" t="n">
         <v>1</v>
@@ -16210,7 +16210,7 @@
         <v>0</v>
       </c>
       <c r="L322" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M322" t="n">
         <v>16</v>
@@ -16327,7 +16327,7 @@
         </is>
       </c>
       <c r="B325" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C325" t="n">
         <v>0</v>
@@ -16348,7 +16348,7 @@
         <v>1</v>
       </c>
       <c r="I325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J325" t="n">
         <v>0</v>
@@ -16357,7 +16357,7 @@
         <v>1</v>
       </c>
       <c r="L325" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M325" t="n">
         <v>20</v>
@@ -16587,10 +16587,10 @@
         <v>1</v>
       </c>
       <c r="G330" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H330" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I330" t="n">
         <v>3</v>
@@ -16602,7 +16602,7 @@
         <v>1</v>
       </c>
       <c r="L330" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M330" t="n">
         <v>58</v>
@@ -16633,7 +16633,7 @@
         <v>12</v>
       </c>
       <c r="F331" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G331" t="n">
         <v>7</v>
@@ -16651,7 +16651,7 @@
         <v>0</v>
       </c>
       <c r="L331" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M331" t="n">
         <v>118</v>
@@ -16670,7 +16670,7 @@
         </is>
       </c>
       <c r="B332" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C332" t="n">
         <v>0</v>
@@ -16700,7 +16700,7 @@
         <v>0</v>
       </c>
       <c r="L332" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M332" t="n">
         <v>45</v>
@@ -17656,7 +17656,7 @@
         <v>0</v>
       </c>
       <c r="D352" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E352" t="n">
         <v>1</v>
@@ -17680,7 +17680,7 @@
         <v>0</v>
       </c>
       <c r="L352" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M352" t="n">
         <v>46</v>
@@ -17754,7 +17754,7 @@
         <v>0</v>
       </c>
       <c r="D354" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E354" t="n">
         <v>2</v>
@@ -17778,7 +17778,7 @@
         <v>0</v>
       </c>
       <c r="L354" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M354" t="n">
         <v>41</v>
@@ -17803,7 +17803,7 @@
         <v>0</v>
       </c>
       <c r="D355" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E355" t="n">
         <v>0</v>
@@ -17827,7 +17827,7 @@
         <v>1</v>
       </c>
       <c r="L355" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M355" t="n">
         <v>23</v>
@@ -17852,7 +17852,7 @@
         <v>0</v>
       </c>
       <c r="D356" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E356" t="n">
         <v>0</v>
@@ -17861,13 +17861,13 @@
         <v>0</v>
       </c>
       <c r="G356" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H356" t="n">
         <v>4</v>
       </c>
       <c r="I356" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J356" t="n">
         <v>2</v>
@@ -17876,7 +17876,7 @@
         <v>0</v>
       </c>
       <c r="L356" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="M356" t="n">
         <v>44</v>
@@ -17956,16 +17956,16 @@
         <v>12</v>
       </c>
       <c r="F358" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G358" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H358" t="n">
         <v>6</v>
       </c>
       <c r="I358" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J358" t="n">
         <v>3</v>
@@ -17974,7 +17974,7 @@
         <v>0</v>
       </c>
       <c r="L358" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="M358" t="n">
         <v>125</v>
@@ -17999,7 +17999,7 @@
         <v>1</v>
       </c>
       <c r="D359" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E359" t="n">
         <v>5</v>
@@ -18023,7 +18023,7 @@
         <v>0</v>
       </c>
       <c r="L359" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M359" t="n">
         <v>91</v>
@@ -18195,7 +18195,7 @@
         <v>0</v>
       </c>
       <c r="D363" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E363" t="n">
         <v>0</v>
@@ -18219,7 +18219,7 @@
         <v>0</v>
       </c>
       <c r="L363" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M363" t="n">
         <v>9</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 20:55
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -6208,7 +6208,7 @@
         <v>0</v>
       </c>
       <c r="D100">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E100">
         <v>2</v>
@@ -6232,7 +6232,7 @@
         <v>0</v>
       </c>
       <c r="L100">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M100">
         <v>19</v>
@@ -7430,7 +7430,7 @@
         <v>2</v>
       </c>
       <c r="D126">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E126">
         <v>6</v>
@@ -7454,7 +7454,7 @@
         <v>0</v>
       </c>
       <c r="L126">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M126">
         <v>55</v>
@@ -12741,7 +12741,7 @@
         <v>3</v>
       </c>
       <c r="D239">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E239">
         <v>46</v>
@@ -12765,7 +12765,7 @@
         <v>0</v>
       </c>
       <c r="L239">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M239">
         <v>185</v>
@@ -14148,7 +14148,7 @@
         <v>1</v>
       </c>
       <c r="C269">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D269">
         <v>2</v>
@@ -14175,7 +14175,7 @@
         <v>0</v>
       </c>
       <c r="L269">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M269">
         <v>48</v>
@@ -14245,7 +14245,7 @@
         <v>6</v>
       </c>
       <c r="D271">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E271">
         <v>21</v>
@@ -14269,7 +14269,7 @@
         <v>0</v>
       </c>
       <c r="L271">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M271">
         <v>184</v>
@@ -14286,7 +14286,7 @@
         <v>285</v>
       </c>
       <c r="B272">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C272">
         <v>10</v>
@@ -14316,7 +14316,7 @@
         <v>1</v>
       </c>
       <c r="L272">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M272">
         <v>251</v>
@@ -14521,7 +14521,7 @@
         <v>290</v>
       </c>
       <c r="B277">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C277">
         <v>2</v>
@@ -14551,7 +14551,7 @@
         <v>1</v>
       </c>
       <c r="L277">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M277">
         <v>132</v>
@@ -14668,7 +14668,7 @@
         <v>2</v>
       </c>
       <c r="D280">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E280">
         <v>8</v>
@@ -14692,7 +14692,7 @@
         <v>0</v>
       </c>
       <c r="L280">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M280">
         <v>87</v>
@@ -14803,7 +14803,7 @@
         <v>296</v>
       </c>
       <c r="B283">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C283">
         <v>12</v>
@@ -14812,7 +14812,7 @@
         <v>22</v>
       </c>
       <c r="E283">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F283">
         <v>13</v>
@@ -14833,7 +14833,7 @@
         <v>1</v>
       </c>
       <c r="L283">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M283">
         <v>272</v>
@@ -14991,7 +14991,7 @@
         <v>300</v>
       </c>
       <c r="B287">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C287">
         <v>11</v>
@@ -15021,7 +15021,7 @@
         <v>0</v>
       </c>
       <c r="L287">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M287">
         <v>283</v>
@@ -15044,7 +15044,7 @@
         <v>4</v>
       </c>
       <c r="D288">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E288">
         <v>24</v>
@@ -15068,7 +15068,7 @@
         <v>1</v>
       </c>
       <c r="L288">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M288">
         <v>101</v>
@@ -15508,7 +15508,7 @@
         <v>311</v>
       </c>
       <c r="B298">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C298">
         <v>0</v>
@@ -15538,7 +15538,7 @@
         <v>4</v>
       </c>
       <c r="L298">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M298">
         <v>140</v>
@@ -15561,7 +15561,7 @@
         <v>0</v>
       </c>
       <c r="D299">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E299">
         <v>2</v>
@@ -15585,7 +15585,7 @@
         <v>0</v>
       </c>
       <c r="L299">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M299">
         <v>25</v>
@@ -15608,7 +15608,7 @@
         <v>0</v>
       </c>
       <c r="D300">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E300">
         <v>7</v>
@@ -15632,7 +15632,7 @@
         <v>0</v>
       </c>
       <c r="L300">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M300">
         <v>50</v>
@@ -15649,22 +15649,22 @@
         <v>314</v>
       </c>
       <c r="B301">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C301">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D301">
         <v>2</v>
       </c>
       <c r="E301">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F301">
         <v>6</v>
       </c>
       <c r="G301">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H301">
         <v>5</v>
@@ -15679,7 +15679,7 @@
         <v>2</v>
       </c>
       <c r="L301">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M301">
         <v>68</v>
@@ -15743,7 +15743,7 @@
         <v>316</v>
       </c>
       <c r="B303">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C303">
         <v>0</v>
@@ -15773,7 +15773,7 @@
         <v>1</v>
       </c>
       <c r="L303">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M303">
         <v>9</v>
@@ -15978,7 +15978,7 @@
         <v>321</v>
       </c>
       <c r="B308">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C308">
         <v>3</v>
@@ -16008,7 +16008,7 @@
         <v>1</v>
       </c>
       <c r="L308">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M308">
         <v>220</v>
@@ -16125,10 +16125,10 @@
         <v>1</v>
       </c>
       <c r="D311">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E311">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F311">
         <v>11</v>
@@ -16149,7 +16149,7 @@
         <v>1</v>
       </c>
       <c r="L311">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M311">
         <v>54</v>
@@ -16172,7 +16172,7 @@
         <v>1</v>
       </c>
       <c r="D312">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E312">
         <v>13</v>
@@ -16196,7 +16196,7 @@
         <v>0</v>
       </c>
       <c r="L312">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M312">
         <v>77</v>
@@ -16213,7 +16213,7 @@
         <v>326</v>
       </c>
       <c r="B313">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C313">
         <v>3</v>
@@ -16243,7 +16243,7 @@
         <v>0</v>
       </c>
       <c r="L313">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M313">
         <v>74</v>
@@ -16354,13 +16354,13 @@
         <v>329</v>
       </c>
       <c r="B316">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C316">
         <v>1</v>
       </c>
       <c r="D316">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E316">
         <v>4</v>
@@ -16369,7 +16369,7 @@
         <v>2</v>
       </c>
       <c r="G316">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H316">
         <v>1</v>
@@ -16384,7 +16384,7 @@
         <v>1</v>
       </c>
       <c r="L316">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M316">
         <v>25</v>
@@ -16495,7 +16495,7 @@
         <v>332</v>
       </c>
       <c r="B319">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C319">
         <v>0</v>
@@ -16525,7 +16525,7 @@
         <v>0</v>
       </c>
       <c r="L319">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M319">
         <v>12</v>
@@ -18951,7 +18951,7 @@
         <v>25</v>
       </c>
       <c r="F371">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G371">
         <v>40</v>
@@ -18969,7 +18969,7 @@
         <v>1</v>
       </c>
       <c r="L371">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M371">
         <v>128</v>
@@ -19095,7 +19095,7 @@
         <v>39</v>
       </c>
       <c r="G374">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H374">
         <v>19</v>
@@ -19110,7 +19110,7 @@
         <v>4</v>
       </c>
       <c r="L374">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M374">
         <v>224</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 21:41
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -18948,13 +18948,13 @@
         <v>6</v>
       </c>
       <c r="E371">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F371">
         <v>24</v>
       </c>
       <c r="G371">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H371">
         <v>13</v>
@@ -18969,7 +18969,7 @@
         <v>1</v>
       </c>
       <c r="L371">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M371">
         <v>128</v>
@@ -19001,7 +19001,7 @@
         <v>3</v>
       </c>
       <c r="G372">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H372">
         <v>9</v>
@@ -19016,7 +19016,7 @@
         <v>0</v>
       </c>
       <c r="L372">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M372">
         <v>72</v>
@@ -19089,13 +19089,13 @@
         <v>9</v>
       </c>
       <c r="E374">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F374">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G374">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="H374">
         <v>19</v>
@@ -19110,7 +19110,7 @@
         <v>4</v>
       </c>
       <c r="L374">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="M374">
         <v>224</v>
@@ -19174,7 +19174,7 @@
         <v>389</v>
       </c>
       <c r="B376">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C376">
         <v>9</v>
@@ -19189,7 +19189,7 @@
         <v>43</v>
       </c>
       <c r="G376">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H376">
         <v>11</v>
@@ -19204,7 +19204,7 @@
         <v>1</v>
       </c>
       <c r="L376">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M376">
         <v>262</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-26 08:05
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -19292,7 +19292,7 @@
         <v>14</v>
       </c>
       <c r="E378">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F378">
         <v>21</v>
@@ -19313,7 +19313,7 @@
         <v>0</v>
       </c>
       <c r="L378">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M378">
         <v>212</v>
@@ -19392,7 +19392,7 @@
         <v>13</v>
       </c>
       <c r="G380">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H380">
         <v>7</v>
@@ -19407,7 +19407,7 @@
         <v>1</v>
       </c>
       <c r="L380">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M380">
         <v>125</v>

</xml_diff>